<commit_message>
adding mean of second algorithm and edit excel errors
</commit_message>
<xml_diff>
--- a/Python/data.xlsx
+++ b/Python/data.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Math. Software\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\mathematics_softwares_project\Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A806BC4-41DF-4665-86B9-4416974CF602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5650" yWindow="0" windowWidth="23040" windowHeight="9800"/>
+    <workbookView xWindow="276" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -53,18 +54,18 @@
     <t>600KB</t>
   </si>
   <si>
-    <t xml:space="preserve"> Run time for different data size</t>
+    <t>Run time for different data size</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -373,20 +374,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M192"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="54" customWidth="1"/>
-    <col min="2" max="2" width="12.90625" customWidth="1"/>
+    <col min="2" max="2" width="12.8984375" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="16.36328125" customWidth="1"/>
-    <col min="11" max="11" width="40.36328125" customWidth="1"/>
-    <col min="12" max="12" width="11.36328125" customWidth="1"/>
-    <col min="13" max="13" width="10.453125" customWidth="1"/>
+    <col min="4" max="4" width="16.3984375" customWidth="1"/>
+    <col min="11" max="11" width="40.3984375" customWidth="1"/>
+    <col min="12" max="12" width="11.3984375" customWidth="1"/>
+    <col min="13" max="13" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -403,7 +404,7 @@
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -420,7 +421,7 @@
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -437,7 +438,7 @@
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -454,7 +455,7 @@
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -471,7 +472,7 @@
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -488,7 +489,7 @@
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -505,7 +506,7 @@
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -513,7 +514,7 @@
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -521,7 +522,7 @@
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -529,7 +530,7 @@
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -537,7 +538,7 @@
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -545,7 +546,7 @@
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -553,7 +554,7 @@
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -562,7 +563,7 @@
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -571,7 +572,7 @@
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -580,7 +581,7 @@
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -589,7 +590,7 @@
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -598,7 +599,7 @@
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -607,7 +608,7 @@
       <c r="L19" s="1"/>
       <c r="M19" s="1"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -615,7 +616,7 @@
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -623,7 +624,7 @@
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -631,7 +632,7 @@
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -639,7 +640,7 @@
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -647,7 +648,7 @@
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -655,7 +656,7 @@
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -664,7 +665,7 @@
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -673,7 +674,7 @@
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -682,7 +683,7 @@
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -691,7 +692,7 @@
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -700,7 +701,7 @@
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -709,7 +710,7 @@
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -717,7 +718,7 @@
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -725,7 +726,7 @@
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -733,7 +734,7 @@
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -741,7 +742,7 @@
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -749,7 +750,7 @@
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -757,7 +758,7 @@
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -765,7 +766,7 @@
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -773,7 +774,7 @@
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -781,7 +782,7 @@
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -789,7 +790,7 @@
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -797,7 +798,7 @@
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -805,7 +806,7 @@
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -813,7 +814,7 @@
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -821,7 +822,7 @@
       <c r="L45" s="1"/>
       <c r="M45" s="1"/>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -829,7 +830,7 @@
       <c r="L46" s="1"/>
       <c r="M46" s="1"/>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -837,7 +838,7 @@
       <c r="L47" s="1"/>
       <c r="M47" s="1"/>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -845,7 +846,7 @@
       <c r="L48" s="1"/>
       <c r="M48" s="1"/>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -853,7 +854,7 @@
       <c r="L49" s="1"/>
       <c r="M49" s="1"/>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -861,7 +862,7 @@
       <c r="L50" s="1"/>
       <c r="M50" s="1"/>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
@@ -869,7 +870,7 @@
       <c r="L51" s="1"/>
       <c r="M51" s="1"/>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -877,7 +878,7 @@
       <c r="L52" s="1"/>
       <c r="M52" s="1"/>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -885,7 +886,7 @@
       <c r="L53" s="1"/>
       <c r="M53" s="1"/>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -893,7 +894,7 @@
       <c r="L54" s="1"/>
       <c r="M54" s="1"/>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -901,7 +902,7 @@
       <c r="L55" s="1"/>
       <c r="M55" s="1"/>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
@@ -909,7 +910,7 @@
       <c r="L56" s="1"/>
       <c r="M56" s="1"/>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -917,7 +918,7 @@
       <c r="L57" s="1"/>
       <c r="M57" s="1"/>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
@@ -925,7 +926,7 @@
       <c r="L58" s="1"/>
       <c r="M58" s="1"/>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
@@ -933,7 +934,7 @@
       <c r="L59" s="1"/>
       <c r="M59" s="1"/>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
@@ -941,7 +942,7 @@
       <c r="L60" s="1"/>
       <c r="M60" s="1"/>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
@@ -949,657 +950,657 @@
       <c r="L61" s="1"/>
       <c r="M61" s="1"/>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="1"/>
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="1"/>
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="1"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="1"/>
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="1"/>
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="1"/>
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="1"/>
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
       <c r="C83" s="1"/>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" s="1"/>
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" s="1"/>
       <c r="B86" s="1"/>
       <c r="C86" s="1"/>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="1"/>
       <c r="B87" s="1"/>
       <c r="C87" s="1"/>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="1"/>
       <c r="B88" s="1"/>
       <c r="C88" s="1"/>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="1"/>
       <c r="B89" s="1"/>
       <c r="C89" s="1"/>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="1"/>
       <c r="B90" s="1"/>
       <c r="C90" s="1"/>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="1"/>
       <c r="B91" s="1"/>
       <c r="C91" s="1"/>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="1"/>
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="1"/>
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" s="1"/>
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="1"/>
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" s="1"/>
       <c r="B97" s="1"/>
       <c r="C97" s="1"/>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" s="1"/>
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" s="1"/>
       <c r="B99" s="1"/>
       <c r="C99" s="1"/>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" s="1"/>
       <c r="B100" s="1"/>
       <c r="C100" s="1"/>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" s="1"/>
       <c r="B101" s="1"/>
       <c r="C101" s="1"/>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" s="1"/>
       <c r="B102" s="1"/>
       <c r="C102" s="1"/>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" s="1"/>
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" s="1"/>
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" s="1"/>
       <c r="B105" s="1"/>
       <c r="C105" s="1"/>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" s="1"/>
       <c r="B106" s="1"/>
       <c r="C106" s="1"/>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" s="1"/>
       <c r="B107" s="1"/>
       <c r="C107" s="1"/>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" s="1"/>
       <c r="B108" s="1"/>
       <c r="C108" s="1"/>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" s="1"/>
       <c r="B109" s="1"/>
       <c r="C109" s="1"/>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" s="1"/>
       <c r="B111" s="1"/>
       <c r="C111" s="1"/>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" s="1"/>
       <c r="B112" s="1"/>
       <c r="C112" s="1"/>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" s="1"/>
       <c r="B113" s="1"/>
       <c r="C113" s="1"/>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" s="1"/>
       <c r="B114" s="1"/>
       <c r="C114" s="1"/>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" s="1"/>
       <c r="B115" s="1"/>
       <c r="C115" s="1"/>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" s="1"/>
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" s="1"/>
       <c r="B117" s="1"/>
       <c r="C117" s="1"/>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" s="1"/>
       <c r="B118" s="1"/>
       <c r="C118" s="1"/>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" s="1"/>
       <c r="B119" s="1"/>
       <c r="C119" s="1"/>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" s="1"/>
       <c r="B120" s="1"/>
       <c r="C120" s="1"/>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" s="1"/>
       <c r="B121" s="1"/>
       <c r="C121" s="1"/>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" s="1"/>
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" s="1"/>
       <c r="B123" s="1"/>
       <c r="C123" s="1"/>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" s="1"/>
       <c r="B124" s="1"/>
       <c r="C124" s="1"/>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" s="1"/>
       <c r="B125" s="1"/>
       <c r="C125" s="1"/>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" s="1"/>
       <c r="B126" s="1"/>
       <c r="C126" s="1"/>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" s="1"/>
       <c r="B127" s="1"/>
       <c r="C127" s="1"/>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" s="1"/>
       <c r="B128" s="1"/>
       <c r="C128" s="1"/>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" s="1"/>
       <c r="B129" s="1"/>
       <c r="C129" s="1"/>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" s="1"/>
       <c r="B130" s="1"/>
       <c r="C130" s="1"/>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" s="1"/>
       <c r="B131" s="1"/>
       <c r="C131" s="1"/>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" s="1"/>
       <c r="B132" s="1"/>
       <c r="C132" s="1"/>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" s="1"/>
       <c r="B133" s="1"/>
       <c r="C133" s="1"/>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" s="1"/>
       <c r="B134" s="1"/>
       <c r="C134" s="1"/>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" s="1"/>
       <c r="B135" s="1"/>
       <c r="C135" s="1"/>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" s="1"/>
       <c r="B136" s="1"/>
       <c r="C136" s="1"/>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" s="1"/>
       <c r="B137" s="1"/>
       <c r="C137" s="1"/>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" s="1"/>
       <c r="B138" s="1"/>
       <c r="C138" s="1"/>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" s="1"/>
       <c r="B139" s="1"/>
       <c r="C139" s="1"/>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" s="1"/>
       <c r="B140" s="1"/>
       <c r="C140" s="1"/>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" s="1"/>
       <c r="B141" s="1"/>
       <c r="C141" s="1"/>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" s="1"/>
       <c r="B142" s="1"/>
       <c r="C142" s="1"/>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" s="1"/>
       <c r="B143" s="1"/>
       <c r="C143" s="1"/>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" s="1"/>
       <c r="B144" s="1"/>
       <c r="C144" s="1"/>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" s="1"/>
       <c r="B145" s="1"/>
       <c r="C145" s="1"/>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" s="1"/>
       <c r="B146" s="1"/>
       <c r="C146" s="1"/>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" s="1"/>
       <c r="B147" s="1"/>
       <c r="C147" s="1"/>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" s="1"/>
       <c r="B148" s="1"/>
       <c r="C148" s="1"/>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" s="1"/>
       <c r="B149" s="1"/>
       <c r="C149" s="1"/>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" s="1"/>
       <c r="B150" s="1"/>
       <c r="C150" s="1"/>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" s="1"/>
       <c r="B151" s="1"/>
       <c r="C151" s="1"/>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" s="1"/>
       <c r="B152" s="1"/>
       <c r="C152" s="1"/>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" s="1"/>
       <c r="B153" s="1"/>
       <c r="C153" s="1"/>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" s="1"/>
       <c r="B154" s="1"/>
       <c r="C154" s="1"/>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" s="1"/>
       <c r="B155" s="1"/>
       <c r="C155" s="1"/>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" s="1"/>
       <c r="B156" s="1"/>
       <c r="C156" s="1"/>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" s="1"/>
       <c r="B157" s="1"/>
       <c r="C157" s="1"/>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" s="1"/>
       <c r="B158" s="1"/>
       <c r="C158" s="1"/>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" s="1"/>
       <c r="B159" s="1"/>
       <c r="C159" s="1"/>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" s="1"/>
       <c r="B160" s="1"/>
       <c r="C160" s="1"/>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" s="1"/>
       <c r="B161" s="1"/>
       <c r="C161" s="1"/>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" s="1"/>
       <c r="B162" s="1"/>
       <c r="C162" s="1"/>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" s="1"/>
       <c r="B163" s="1"/>
       <c r="C163" s="1"/>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" s="1"/>
       <c r="B164" s="1"/>
       <c r="C164" s="1"/>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" s="1"/>
       <c r="B165" s="1"/>
       <c r="C165" s="1"/>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" s="1"/>
       <c r="B166" s="1"/>
       <c r="C166" s="1"/>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" s="1"/>
       <c r="B167" s="1"/>
       <c r="C167" s="1"/>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" s="1"/>
       <c r="B168" s="1"/>
       <c r="C168" s="1"/>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" s="1"/>
       <c r="B169" s="1"/>
       <c r="C169" s="1"/>
     </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" s="1"/>
       <c r="B170" s="1"/>
       <c r="C170" s="1"/>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" s="1"/>
       <c r="B171" s="1"/>
       <c r="C171" s="1"/>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" s="1"/>
       <c r="B172" s="1"/>
       <c r="C172" s="1"/>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" s="1"/>
       <c r="B173" s="1"/>
       <c r="C173" s="1"/>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" s="1"/>
       <c r="B174" s="1"/>
       <c r="C174" s="1"/>
     </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" s="1"/>
       <c r="B175" s="1"/>
       <c r="C175" s="1"/>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" s="1"/>
       <c r="B176" s="1"/>
       <c r="C176" s="1"/>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="1"/>
       <c r="B177" s="1"/>
       <c r="C177" s="1"/>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="1"/>
       <c r="B178" s="1"/>
       <c r="C178" s="1"/>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="1"/>
       <c r="B179" s="1"/>
       <c r="C179" s="1"/>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="1"/>
       <c r="B180" s="1"/>
       <c r="C180" s="1"/>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="1"/>
       <c r="B181" s="1"/>
       <c r="C181" s="1"/>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="1"/>
       <c r="B182" s="1"/>
       <c r="C182" s="1"/>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="1"/>
       <c r="B183" s="1"/>
       <c r="C183" s="1"/>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="1"/>
       <c r="B184" s="1"/>
       <c r="C184" s="1"/>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="1"/>
       <c r="B185" s="1"/>
       <c r="C185" s="1"/>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="1"/>
       <c r="B186" s="1"/>
       <c r="C186" s="1"/>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="1"/>
       <c r="B187" s="1"/>
       <c r="C187" s="1"/>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="1"/>
       <c r="B188" s="1"/>
       <c r="C188" s="1"/>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="1"/>
       <c r="B189" s="1"/>
       <c r="C189" s="1"/>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="1"/>
       <c r="B190" s="1"/>
       <c r="C190" s="1"/>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="1"/>
       <c r="B191" s="1"/>
       <c r="C191" s="1"/>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="1"/>
       <c r="B192" s="1"/>
       <c r="C192" s="1"/>

</xml_diff>